<commit_message>
feat(pkl): absensi PKL, dashboard Kaprodi & kaitan DUDI-program
- tabel pkl_attendance + RLS (DUDI tulis siswanya, Kaprodi/staf baca, admin delete)
- RLS observasi: izinkan DUDI menulis observasi siswa PKL-nya
- dashboard Kaprodi (kaprodi/): ringkasan PKL, mitra DUDI, rekap absensi, observasi DUDI
- template DUDI: kolom kode_program menautkan DUDI ke program/Kaprodi (wizard + setup-wizard + edge fn)
- api.js: pkl_attendance masuk cascade-delete siswa

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/file uji/template_dudi.xlsx
+++ b/file uji/template_dudi.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="DATA" sheetId="1" r:id="rId1"/>
+    <sheet name="PETUNJUK" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B301"/>
+  <dimension ref="A1:C301"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -407,6 +408,9 @@
       <c r="B1" s="1" t="str">
         <v>nama_penanggung_jawab</v>
       </c>
+      <c r="C1" s="1" t="str">
+        <v>kode_program</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
@@ -415,6 +419,9 @@
       <c r="B2" s="1" t="str">
         <v>Hendra Setiawan</v>
       </c>
+      <c r="C2" s="1" t="str">
+        <v>TKJ</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
@@ -423,6 +430,9 @@
       <c r="B3" s="1" t="str">
         <v>Yulia Permatasari</v>
       </c>
+      <c r="C3" s="1" t="str">
+        <v>TKJ</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
@@ -431,6 +441,9 @@
       <c r="B4" s="1" t="str">
         <v/>
       </c>
+      <c r="C4" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
@@ -439,6 +452,9 @@
       <c r="B5" s="1" t="str">
         <v/>
       </c>
+      <c r="C5" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
@@ -447,6 +463,9 @@
       <c r="B6" s="1" t="str">
         <v/>
       </c>
+      <c r="C6" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="str">
@@ -455,6 +474,9 @@
       <c r="B7" s="1" t="str">
         <v/>
       </c>
+      <c r="C7" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="str">
@@ -463,6 +485,9 @@
       <c r="B8" s="1" t="str">
         <v/>
       </c>
+      <c r="C8" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="str">
@@ -471,6 +496,9 @@
       <c r="B9" s="1" t="str">
         <v/>
       </c>
+      <c r="C9" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="str">
@@ -479,6 +507,9 @@
       <c r="B10" s="1" t="str">
         <v/>
       </c>
+      <c r="C10" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="str">
@@ -487,6 +518,9 @@
       <c r="B11" s="1" t="str">
         <v/>
       </c>
+      <c r="C11" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="str">
@@ -495,6 +529,9 @@
       <c r="B12" s="1" t="str">
         <v/>
       </c>
+      <c r="C12" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="str">
@@ -503,6 +540,9 @@
       <c r="B13" s="1" t="str">
         <v/>
       </c>
+      <c r="C13" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="str">
@@ -511,6 +551,9 @@
       <c r="B14" s="1" t="str">
         <v/>
       </c>
+      <c r="C14" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="str">
@@ -519,6 +562,9 @@
       <c r="B15" s="1" t="str">
         <v/>
       </c>
+      <c r="C15" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="str">
@@ -527,6 +573,9 @@
       <c r="B16" s="1" t="str">
         <v/>
       </c>
+      <c r="C16" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="str">
@@ -535,6 +584,9 @@
       <c r="B17" s="1" t="str">
         <v/>
       </c>
+      <c r="C17" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="str">
@@ -543,6 +595,9 @@
       <c r="B18" s="1" t="str">
         <v/>
       </c>
+      <c r="C18" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="str">
@@ -551,6 +606,9 @@
       <c r="B19" s="1" t="str">
         <v/>
       </c>
+      <c r="C19" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="str">
@@ -559,6 +617,9 @@
       <c r="B20" s="1" t="str">
         <v/>
       </c>
+      <c r="C20" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="str">
@@ -567,6 +628,9 @@
       <c r="B21" s="1" t="str">
         <v/>
       </c>
+      <c r="C21" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="str">
@@ -575,6 +639,9 @@
       <c r="B22" s="1" t="str">
         <v/>
       </c>
+      <c r="C22" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="str">
@@ -583,6 +650,9 @@
       <c r="B23" s="1" t="str">
         <v/>
       </c>
+      <c r="C23" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="str">
@@ -591,6 +661,9 @@
       <c r="B24" s="1" t="str">
         <v/>
       </c>
+      <c r="C24" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="str">
@@ -599,6 +672,9 @@
       <c r="B25" s="1" t="str">
         <v/>
       </c>
+      <c r="C25" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="str">
@@ -607,6 +683,9 @@
       <c r="B26" s="1" t="str">
         <v/>
       </c>
+      <c r="C26" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="str">
@@ -615,6 +694,9 @@
       <c r="B27" s="1" t="str">
         <v/>
       </c>
+      <c r="C27" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="str">
@@ -623,6 +705,9 @@
       <c r="B28" s="1" t="str">
         <v/>
       </c>
+      <c r="C28" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="str">
@@ -631,6 +716,9 @@
       <c r="B29" s="1" t="str">
         <v/>
       </c>
+      <c r="C29" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="str">
@@ -639,6 +727,9 @@
       <c r="B30" s="1" t="str">
         <v/>
       </c>
+      <c r="C30" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="str">
@@ -647,6 +738,9 @@
       <c r="B31" s="1" t="str">
         <v/>
       </c>
+      <c r="C31" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="str">
@@ -655,6 +749,9 @@
       <c r="B32" s="1" t="str">
         <v/>
       </c>
+      <c r="C32" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="str">
@@ -663,6 +760,9 @@
       <c r="B33" s="1" t="str">
         <v/>
       </c>
+      <c r="C33" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="str">
@@ -671,6 +771,9 @@
       <c r="B34" s="1" t="str">
         <v/>
       </c>
+      <c r="C34" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="str">
@@ -679,6 +782,9 @@
       <c r="B35" s="1" t="str">
         <v/>
       </c>
+      <c r="C35" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="str">
@@ -687,6 +793,9 @@
       <c r="B36" s="1" t="str">
         <v/>
       </c>
+      <c r="C36" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="str">
@@ -695,6 +804,9 @@
       <c r="B37" s="1" t="str">
         <v/>
       </c>
+      <c r="C37" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="str">
@@ -703,6 +815,9 @@
       <c r="B38" s="1" t="str">
         <v/>
       </c>
+      <c r="C38" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="str">
@@ -711,6 +826,9 @@
       <c r="B39" s="1" t="str">
         <v/>
       </c>
+      <c r="C39" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="str">
@@ -719,6 +837,9 @@
       <c r="B40" s="1" t="str">
         <v/>
       </c>
+      <c r="C40" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="str">
@@ -727,6 +848,9 @@
       <c r="B41" s="1" t="str">
         <v/>
       </c>
+      <c r="C41" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="str">
@@ -735,6 +859,9 @@
       <c r="B42" s="1" t="str">
         <v/>
       </c>
+      <c r="C42" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="str">
@@ -743,6 +870,9 @@
       <c r="B43" s="1" t="str">
         <v/>
       </c>
+      <c r="C43" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="str">
@@ -751,6 +881,9 @@
       <c r="B44" s="1" t="str">
         <v/>
       </c>
+      <c r="C44" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="str">
@@ -759,6 +892,9 @@
       <c r="B45" s="1" t="str">
         <v/>
       </c>
+      <c r="C45" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="str">
@@ -767,6 +903,9 @@
       <c r="B46" s="1" t="str">
         <v/>
       </c>
+      <c r="C46" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="str">
@@ -775,6 +914,9 @@
       <c r="B47" s="1" t="str">
         <v/>
       </c>
+      <c r="C47" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="str">
@@ -783,6 +925,9 @@
       <c r="B48" s="1" t="str">
         <v/>
       </c>
+      <c r="C48" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="str">
@@ -791,6 +936,9 @@
       <c r="B49" s="1" t="str">
         <v/>
       </c>
+      <c r="C49" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="str">
@@ -799,6 +947,9 @@
       <c r="B50" s="1" t="str">
         <v/>
       </c>
+      <c r="C50" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="str">
@@ -807,6 +958,9 @@
       <c r="B51" s="1" t="str">
         <v/>
       </c>
+      <c r="C51" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="str">
@@ -815,6 +969,9 @@
       <c r="B52" s="1" t="str">
         <v/>
       </c>
+      <c r="C52" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="str">
@@ -823,6 +980,9 @@
       <c r="B53" s="1" t="str">
         <v/>
       </c>
+      <c r="C53" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="str">
@@ -831,6 +991,9 @@
       <c r="B54" s="1" t="str">
         <v/>
       </c>
+      <c r="C54" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="str">
@@ -839,6 +1002,9 @@
       <c r="B55" s="1" t="str">
         <v/>
       </c>
+      <c r="C55" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="str">
@@ -847,6 +1013,9 @@
       <c r="B56" s="1" t="str">
         <v/>
       </c>
+      <c r="C56" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="str">
@@ -855,6 +1024,9 @@
       <c r="B57" s="1" t="str">
         <v/>
       </c>
+      <c r="C57" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="str">
@@ -863,6 +1035,9 @@
       <c r="B58" s="1" t="str">
         <v/>
       </c>
+      <c r="C58" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="str">
@@ -871,6 +1046,9 @@
       <c r="B59" s="1" t="str">
         <v/>
       </c>
+      <c r="C59" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="str">
@@ -879,6 +1057,9 @@
       <c r="B60" s="1" t="str">
         <v/>
       </c>
+      <c r="C60" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="str">
@@ -887,6 +1068,9 @@
       <c r="B61" s="1" t="str">
         <v/>
       </c>
+      <c r="C61" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="str">
@@ -895,6 +1079,9 @@
       <c r="B62" s="1" t="str">
         <v/>
       </c>
+      <c r="C62" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="str">
@@ -903,6 +1090,9 @@
       <c r="B63" s="1" t="str">
         <v/>
       </c>
+      <c r="C63" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="str">
@@ -911,6 +1101,9 @@
       <c r="B64" s="1" t="str">
         <v/>
       </c>
+      <c r="C64" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="str">
@@ -919,6 +1112,9 @@
       <c r="B65" s="1" t="str">
         <v/>
       </c>
+      <c r="C65" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="str">
@@ -927,6 +1123,9 @@
       <c r="B66" s="1" t="str">
         <v/>
       </c>
+      <c r="C66" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="str">
@@ -935,6 +1134,9 @@
       <c r="B67" s="1" t="str">
         <v/>
       </c>
+      <c r="C67" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="str">
@@ -943,6 +1145,9 @@
       <c r="B68" s="1" t="str">
         <v/>
       </c>
+      <c r="C68" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="str">
@@ -951,6 +1156,9 @@
       <c r="B69" s="1" t="str">
         <v/>
       </c>
+      <c r="C69" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="str">
@@ -959,6 +1167,9 @@
       <c r="B70" s="1" t="str">
         <v/>
       </c>
+      <c r="C70" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="str">
@@ -967,6 +1178,9 @@
       <c r="B71" s="1" t="str">
         <v/>
       </c>
+      <c r="C71" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="str">
@@ -975,6 +1189,9 @@
       <c r="B72" s="1" t="str">
         <v/>
       </c>
+      <c r="C72" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="str">
@@ -983,6 +1200,9 @@
       <c r="B73" s="1" t="str">
         <v/>
       </c>
+      <c r="C73" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="str">
@@ -991,6 +1211,9 @@
       <c r="B74" s="1" t="str">
         <v/>
       </c>
+      <c r="C74" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="str">
@@ -999,6 +1222,9 @@
       <c r="B75" s="1" t="str">
         <v/>
       </c>
+      <c r="C75" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="str">
@@ -1007,6 +1233,9 @@
       <c r="B76" s="1" t="str">
         <v/>
       </c>
+      <c r="C76" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="str">
@@ -1015,6 +1244,9 @@
       <c r="B77" s="1" t="str">
         <v/>
       </c>
+      <c r="C77" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="str">
@@ -1023,6 +1255,9 @@
       <c r="B78" s="1" t="str">
         <v/>
       </c>
+      <c r="C78" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="str">
@@ -1031,6 +1266,9 @@
       <c r="B79" s="1" t="str">
         <v/>
       </c>
+      <c r="C79" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="str">
@@ -1039,6 +1277,9 @@
       <c r="B80" s="1" t="str">
         <v/>
       </c>
+      <c r="C80" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="str">
@@ -1047,6 +1288,9 @@
       <c r="B81" s="1" t="str">
         <v/>
       </c>
+      <c r="C81" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="str">
@@ -1055,6 +1299,9 @@
       <c r="B82" s="1" t="str">
         <v/>
       </c>
+      <c r="C82" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="str">
@@ -1063,6 +1310,9 @@
       <c r="B83" s="1" t="str">
         <v/>
       </c>
+      <c r="C83" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="str">
@@ -1071,6 +1321,9 @@
       <c r="B84" s="1" t="str">
         <v/>
       </c>
+      <c r="C84" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="str">
@@ -1079,6 +1332,9 @@
       <c r="B85" s="1" t="str">
         <v/>
       </c>
+      <c r="C85" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="str">
@@ -1087,6 +1343,9 @@
       <c r="B86" s="1" t="str">
         <v/>
       </c>
+      <c r="C86" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="str">
@@ -1095,6 +1354,9 @@
       <c r="B87" s="1" t="str">
         <v/>
       </c>
+      <c r="C87" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="str">
@@ -1103,6 +1365,9 @@
       <c r="B88" s="1" t="str">
         <v/>
       </c>
+      <c r="C88" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="str">
@@ -1111,6 +1376,9 @@
       <c r="B89" s="1" t="str">
         <v/>
       </c>
+      <c r="C89" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="str">
@@ -1119,6 +1387,9 @@
       <c r="B90" s="1" t="str">
         <v/>
       </c>
+      <c r="C90" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="str">
@@ -1127,6 +1398,9 @@
       <c r="B91" s="1" t="str">
         <v/>
       </c>
+      <c r="C91" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="str">
@@ -1135,6 +1409,9 @@
       <c r="B92" s="1" t="str">
         <v/>
       </c>
+      <c r="C92" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="str">
@@ -1143,6 +1420,9 @@
       <c r="B93" s="1" t="str">
         <v/>
       </c>
+      <c r="C93" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="str">
@@ -1151,6 +1431,9 @@
       <c r="B94" s="1" t="str">
         <v/>
       </c>
+      <c r="C94" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="str">
@@ -1159,6 +1442,9 @@
       <c r="B95" s="1" t="str">
         <v/>
       </c>
+      <c r="C95" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="str">
@@ -1167,6 +1453,9 @@
       <c r="B96" s="1" t="str">
         <v/>
       </c>
+      <c r="C96" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="str">
@@ -1175,6 +1464,9 @@
       <c r="B97" s="1" t="str">
         <v/>
       </c>
+      <c r="C97" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="str">
@@ -1183,6 +1475,9 @@
       <c r="B98" s="1" t="str">
         <v/>
       </c>
+      <c r="C98" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="str">
@@ -1191,6 +1486,9 @@
       <c r="B99" s="1" t="str">
         <v/>
       </c>
+      <c r="C99" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="str">
@@ -1199,6 +1497,9 @@
       <c r="B100" s="1" t="str">
         <v/>
       </c>
+      <c r="C100" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="str">
@@ -1207,6 +1508,9 @@
       <c r="B101" s="1" t="str">
         <v/>
       </c>
+      <c r="C101" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="str">
@@ -1215,6 +1519,9 @@
       <c r="B102" s="1" t="str">
         <v/>
       </c>
+      <c r="C102" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="str">
@@ -1223,6 +1530,9 @@
       <c r="B103" s="1" t="str">
         <v/>
       </c>
+      <c r="C103" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="str">
@@ -1231,6 +1541,9 @@
       <c r="B104" s="1" t="str">
         <v/>
       </c>
+      <c r="C104" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="str">
@@ -1239,6 +1552,9 @@
       <c r="B105" s="1" t="str">
         <v/>
       </c>
+      <c r="C105" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="str">
@@ -1247,6 +1563,9 @@
       <c r="B106" s="1" t="str">
         <v/>
       </c>
+      <c r="C106" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="str">
@@ -1255,6 +1574,9 @@
       <c r="B107" s="1" t="str">
         <v/>
       </c>
+      <c r="C107" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="str">
@@ -1263,6 +1585,9 @@
       <c r="B108" s="1" t="str">
         <v/>
       </c>
+      <c r="C108" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="str">
@@ -1271,6 +1596,9 @@
       <c r="B109" s="1" t="str">
         <v/>
       </c>
+      <c r="C109" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="str">
@@ -1279,6 +1607,9 @@
       <c r="B110" s="1" t="str">
         <v/>
       </c>
+      <c r="C110" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="str">
@@ -1287,6 +1618,9 @@
       <c r="B111" s="1" t="str">
         <v/>
       </c>
+      <c r="C111" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="str">
@@ -1295,6 +1629,9 @@
       <c r="B112" s="1" t="str">
         <v/>
       </c>
+      <c r="C112" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="str">
@@ -1303,6 +1640,9 @@
       <c r="B113" s="1" t="str">
         <v/>
       </c>
+      <c r="C113" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="str">
@@ -1311,6 +1651,9 @@
       <c r="B114" s="1" t="str">
         <v/>
       </c>
+      <c r="C114" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="str">
@@ -1319,6 +1662,9 @@
       <c r="B115" s="1" t="str">
         <v/>
       </c>
+      <c r="C115" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="str">
@@ -1327,6 +1673,9 @@
       <c r="B116" s="1" t="str">
         <v/>
       </c>
+      <c r="C116" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="str">
@@ -1335,6 +1684,9 @@
       <c r="B117" s="1" t="str">
         <v/>
       </c>
+      <c r="C117" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="str">
@@ -1343,6 +1695,9 @@
       <c r="B118" s="1" t="str">
         <v/>
       </c>
+      <c r="C118" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="str">
@@ -1351,6 +1706,9 @@
       <c r="B119" s="1" t="str">
         <v/>
       </c>
+      <c r="C119" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="str">
@@ -1359,6 +1717,9 @@
       <c r="B120" s="1" t="str">
         <v/>
       </c>
+      <c r="C120" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="str">
@@ -1367,6 +1728,9 @@
       <c r="B121" s="1" t="str">
         <v/>
       </c>
+      <c r="C121" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="str">
@@ -1375,6 +1739,9 @@
       <c r="B122" s="1" t="str">
         <v/>
       </c>
+      <c r="C122" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="str">
@@ -1383,6 +1750,9 @@
       <c r="B123" s="1" t="str">
         <v/>
       </c>
+      <c r="C123" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="str">
@@ -1391,6 +1761,9 @@
       <c r="B124" s="1" t="str">
         <v/>
       </c>
+      <c r="C124" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="str">
@@ -1399,6 +1772,9 @@
       <c r="B125" s="1" t="str">
         <v/>
       </c>
+      <c r="C125" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="str">
@@ -1407,6 +1783,9 @@
       <c r="B126" s="1" t="str">
         <v/>
       </c>
+      <c r="C126" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="str">
@@ -1415,6 +1794,9 @@
       <c r="B127" s="1" t="str">
         <v/>
       </c>
+      <c r="C127" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="str">
@@ -1423,6 +1805,9 @@
       <c r="B128" s="1" t="str">
         <v/>
       </c>
+      <c r="C128" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="str">
@@ -1431,6 +1816,9 @@
       <c r="B129" s="1" t="str">
         <v/>
       </c>
+      <c r="C129" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="str">
@@ -1439,6 +1827,9 @@
       <c r="B130" s="1" t="str">
         <v/>
       </c>
+      <c r="C130" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="str">
@@ -1447,6 +1838,9 @@
       <c r="B131" s="1" t="str">
         <v/>
       </c>
+      <c r="C131" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="str">
@@ -1455,6 +1849,9 @@
       <c r="B132" s="1" t="str">
         <v/>
       </c>
+      <c r="C132" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="str">
@@ -1463,6 +1860,9 @@
       <c r="B133" s="1" t="str">
         <v/>
       </c>
+      <c r="C133" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="str">
@@ -1471,6 +1871,9 @@
       <c r="B134" s="1" t="str">
         <v/>
       </c>
+      <c r="C134" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="str">
@@ -1479,6 +1882,9 @@
       <c r="B135" s="1" t="str">
         <v/>
       </c>
+      <c r="C135" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="str">
@@ -1487,6 +1893,9 @@
       <c r="B136" s="1" t="str">
         <v/>
       </c>
+      <c r="C136" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="str">
@@ -1495,6 +1904,9 @@
       <c r="B137" s="1" t="str">
         <v/>
       </c>
+      <c r="C137" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="str">
@@ -1503,6 +1915,9 @@
       <c r="B138" s="1" t="str">
         <v/>
       </c>
+      <c r="C138" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="str">
@@ -1511,6 +1926,9 @@
       <c r="B139" s="1" t="str">
         <v/>
       </c>
+      <c r="C139" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="str">
@@ -1519,6 +1937,9 @@
       <c r="B140" s="1" t="str">
         <v/>
       </c>
+      <c r="C140" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="str">
@@ -1527,6 +1948,9 @@
       <c r="B141" s="1" t="str">
         <v/>
       </c>
+      <c r="C141" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="str">
@@ -1535,6 +1959,9 @@
       <c r="B142" s="1" t="str">
         <v/>
       </c>
+      <c r="C142" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="str">
@@ -1543,6 +1970,9 @@
       <c r="B143" s="1" t="str">
         <v/>
       </c>
+      <c r="C143" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="str">
@@ -1551,6 +1981,9 @@
       <c r="B144" s="1" t="str">
         <v/>
       </c>
+      <c r="C144" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="str">
@@ -1559,6 +1992,9 @@
       <c r="B145" s="1" t="str">
         <v/>
       </c>
+      <c r="C145" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="str">
@@ -1567,6 +2003,9 @@
       <c r="B146" s="1" t="str">
         <v/>
       </c>
+      <c r="C146" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="str">
@@ -1575,6 +2014,9 @@
       <c r="B147" s="1" t="str">
         <v/>
       </c>
+      <c r="C147" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="str">
@@ -1583,6 +2025,9 @@
       <c r="B148" s="1" t="str">
         <v/>
       </c>
+      <c r="C148" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="str">
@@ -1591,6 +2036,9 @@
       <c r="B149" s="1" t="str">
         <v/>
       </c>
+      <c r="C149" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="str">
@@ -1599,6 +2047,9 @@
       <c r="B150" s="1" t="str">
         <v/>
       </c>
+      <c r="C150" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="str">
@@ -1607,6 +2058,9 @@
       <c r="B151" s="1" t="str">
         <v/>
       </c>
+      <c r="C151" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="str">
@@ -1615,6 +2069,9 @@
       <c r="B152" s="1" t="str">
         <v/>
       </c>
+      <c r="C152" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="str">
@@ -1623,6 +2080,9 @@
       <c r="B153" s="1" t="str">
         <v/>
       </c>
+      <c r="C153" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="str">
@@ -1631,6 +2091,9 @@
       <c r="B154" s="1" t="str">
         <v/>
       </c>
+      <c r="C154" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="str">
@@ -1639,6 +2102,9 @@
       <c r="B155" s="1" t="str">
         <v/>
       </c>
+      <c r="C155" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="str">
@@ -1647,6 +2113,9 @@
       <c r="B156" s="1" t="str">
         <v/>
       </c>
+      <c r="C156" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="str">
@@ -1655,6 +2124,9 @@
       <c r="B157" s="1" t="str">
         <v/>
       </c>
+      <c r="C157" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="str">
@@ -1663,6 +2135,9 @@
       <c r="B158" s="1" t="str">
         <v/>
       </c>
+      <c r="C158" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="str">
@@ -1671,6 +2146,9 @@
       <c r="B159" s="1" t="str">
         <v/>
       </c>
+      <c r="C159" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="str">
@@ -1679,6 +2157,9 @@
       <c r="B160" s="1" t="str">
         <v/>
       </c>
+      <c r="C160" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="str">
@@ -1687,6 +2168,9 @@
       <c r="B161" s="1" t="str">
         <v/>
       </c>
+      <c r="C161" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="str">
@@ -1695,6 +2179,9 @@
       <c r="B162" s="1" t="str">
         <v/>
       </c>
+      <c r="C162" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="str">
@@ -1703,6 +2190,9 @@
       <c r="B163" s="1" t="str">
         <v/>
       </c>
+      <c r="C163" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="str">
@@ -1711,6 +2201,9 @@
       <c r="B164" s="1" t="str">
         <v/>
       </c>
+      <c r="C164" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="str">
@@ -1719,6 +2212,9 @@
       <c r="B165" s="1" t="str">
         <v/>
       </c>
+      <c r="C165" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="str">
@@ -1727,6 +2223,9 @@
       <c r="B166" s="1" t="str">
         <v/>
       </c>
+      <c r="C166" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="str">
@@ -1735,6 +2234,9 @@
       <c r="B167" s="1" t="str">
         <v/>
       </c>
+      <c r="C167" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="str">
@@ -1743,6 +2245,9 @@
       <c r="B168" s="1" t="str">
         <v/>
       </c>
+      <c r="C168" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="str">
@@ -1751,6 +2256,9 @@
       <c r="B169" s="1" t="str">
         <v/>
       </c>
+      <c r="C169" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="str">
@@ -1759,6 +2267,9 @@
       <c r="B170" s="1" t="str">
         <v/>
       </c>
+      <c r="C170" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="str">
@@ -1767,6 +2278,9 @@
       <c r="B171" s="1" t="str">
         <v/>
       </c>
+      <c r="C171" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="str">
@@ -1775,6 +2289,9 @@
       <c r="B172" s="1" t="str">
         <v/>
       </c>
+      <c r="C172" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="str">
@@ -1783,6 +2300,9 @@
       <c r="B173" s="1" t="str">
         <v/>
       </c>
+      <c r="C173" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="str">
@@ -1791,6 +2311,9 @@
       <c r="B174" s="1" t="str">
         <v/>
       </c>
+      <c r="C174" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="str">
@@ -1799,6 +2322,9 @@
       <c r="B175" s="1" t="str">
         <v/>
       </c>
+      <c r="C175" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="str">
@@ -1807,6 +2333,9 @@
       <c r="B176" s="1" t="str">
         <v/>
       </c>
+      <c r="C176" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="str">
@@ -1815,6 +2344,9 @@
       <c r="B177" s="1" t="str">
         <v/>
       </c>
+      <c r="C177" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="str">
@@ -1823,6 +2355,9 @@
       <c r="B178" s="1" t="str">
         <v/>
       </c>
+      <c r="C178" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="str">
@@ -1831,6 +2366,9 @@
       <c r="B179" s="1" t="str">
         <v/>
       </c>
+      <c r="C179" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="str">
@@ -1839,6 +2377,9 @@
       <c r="B180" s="1" t="str">
         <v/>
       </c>
+      <c r="C180" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="str">
@@ -1847,6 +2388,9 @@
       <c r="B181" s="1" t="str">
         <v/>
       </c>
+      <c r="C181" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="str">
@@ -1855,6 +2399,9 @@
       <c r="B182" s="1" t="str">
         <v/>
       </c>
+      <c r="C182" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="str">
@@ -1863,6 +2410,9 @@
       <c r="B183" s="1" t="str">
         <v/>
       </c>
+      <c r="C183" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="str">
@@ -1871,6 +2421,9 @@
       <c r="B184" s="1" t="str">
         <v/>
       </c>
+      <c r="C184" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="str">
@@ -1879,6 +2432,9 @@
       <c r="B185" s="1" t="str">
         <v/>
       </c>
+      <c r="C185" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="str">
@@ -1887,6 +2443,9 @@
       <c r="B186" s="1" t="str">
         <v/>
       </c>
+      <c r="C186" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="str">
@@ -1895,6 +2454,9 @@
       <c r="B187" s="1" t="str">
         <v/>
       </c>
+      <c r="C187" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="str">
@@ -1903,6 +2465,9 @@
       <c r="B188" s="1" t="str">
         <v/>
       </c>
+      <c r="C188" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="str">
@@ -1911,6 +2476,9 @@
       <c r="B189" s="1" t="str">
         <v/>
       </c>
+      <c r="C189" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="str">
@@ -1919,6 +2487,9 @@
       <c r="B190" s="1" t="str">
         <v/>
       </c>
+      <c r="C190" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="str">
@@ -1927,6 +2498,9 @@
       <c r="B191" s="1" t="str">
         <v/>
       </c>
+      <c r="C191" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="str">
@@ -1935,6 +2509,9 @@
       <c r="B192" s="1" t="str">
         <v/>
       </c>
+      <c r="C192" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="str">
@@ -1943,6 +2520,9 @@
       <c r="B193" s="1" t="str">
         <v/>
       </c>
+      <c r="C193" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="str">
@@ -1951,6 +2531,9 @@
       <c r="B194" s="1" t="str">
         <v/>
       </c>
+      <c r="C194" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="str">
@@ -1959,6 +2542,9 @@
       <c r="B195" s="1" t="str">
         <v/>
       </c>
+      <c r="C195" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="str">
@@ -1967,6 +2553,9 @@
       <c r="B196" s="1" t="str">
         <v/>
       </c>
+      <c r="C196" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="str">
@@ -1975,6 +2564,9 @@
       <c r="B197" s="1" t="str">
         <v/>
       </c>
+      <c r="C197" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="str">
@@ -1983,6 +2575,9 @@
       <c r="B198" s="1" t="str">
         <v/>
       </c>
+      <c r="C198" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="str">
@@ -1991,6 +2586,9 @@
       <c r="B199" s="1" t="str">
         <v/>
       </c>
+      <c r="C199" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="str">
@@ -1999,6 +2597,9 @@
       <c r="B200" s="1" t="str">
         <v/>
       </c>
+      <c r="C200" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="str">
@@ -2007,6 +2608,9 @@
       <c r="B201" s="1" t="str">
         <v/>
       </c>
+      <c r="C201" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="str">
@@ -2015,6 +2619,9 @@
       <c r="B202" s="1" t="str">
         <v/>
       </c>
+      <c r="C202" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="str">
@@ -2023,6 +2630,9 @@
       <c r="B203" s="1" t="str">
         <v/>
       </c>
+      <c r="C203" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="str">
@@ -2031,6 +2641,9 @@
       <c r="B204" s="1" t="str">
         <v/>
       </c>
+      <c r="C204" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="str">
@@ -2039,6 +2652,9 @@
       <c r="B205" s="1" t="str">
         <v/>
       </c>
+      <c r="C205" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="str">
@@ -2047,6 +2663,9 @@
       <c r="B206" s="1" t="str">
         <v/>
       </c>
+      <c r="C206" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="str">
@@ -2055,6 +2674,9 @@
       <c r="B207" s="1" t="str">
         <v/>
       </c>
+      <c r="C207" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="str">
@@ -2063,6 +2685,9 @@
       <c r="B208" s="1" t="str">
         <v/>
       </c>
+      <c r="C208" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="str">
@@ -2071,6 +2696,9 @@
       <c r="B209" s="1" t="str">
         <v/>
       </c>
+      <c r="C209" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="str">
@@ -2079,6 +2707,9 @@
       <c r="B210" s="1" t="str">
         <v/>
       </c>
+      <c r="C210" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="str">
@@ -2087,6 +2718,9 @@
       <c r="B211" s="1" t="str">
         <v/>
       </c>
+      <c r="C211" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="str">
@@ -2095,6 +2729,9 @@
       <c r="B212" s="1" t="str">
         <v/>
       </c>
+      <c r="C212" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="str">
@@ -2103,6 +2740,9 @@
       <c r="B213" s="1" t="str">
         <v/>
       </c>
+      <c r="C213" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="str">
@@ -2111,6 +2751,9 @@
       <c r="B214" s="1" t="str">
         <v/>
       </c>
+      <c r="C214" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="str">
@@ -2119,6 +2762,9 @@
       <c r="B215" s="1" t="str">
         <v/>
       </c>
+      <c r="C215" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="str">
@@ -2127,6 +2773,9 @@
       <c r="B216" s="1" t="str">
         <v/>
       </c>
+      <c r="C216" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="str">
@@ -2135,6 +2784,9 @@
       <c r="B217" s="1" t="str">
         <v/>
       </c>
+      <c r="C217" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="str">
@@ -2143,6 +2795,9 @@
       <c r="B218" s="1" t="str">
         <v/>
       </c>
+      <c r="C218" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="str">
@@ -2151,6 +2806,9 @@
       <c r="B219" s="1" t="str">
         <v/>
       </c>
+      <c r="C219" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="str">
@@ -2159,6 +2817,9 @@
       <c r="B220" s="1" t="str">
         <v/>
       </c>
+      <c r="C220" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="str">
@@ -2167,6 +2828,9 @@
       <c r="B221" s="1" t="str">
         <v/>
       </c>
+      <c r="C221" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="str">
@@ -2175,6 +2839,9 @@
       <c r="B222" s="1" t="str">
         <v/>
       </c>
+      <c r="C222" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="str">
@@ -2183,6 +2850,9 @@
       <c r="B223" s="1" t="str">
         <v/>
       </c>
+      <c r="C223" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="str">
@@ -2191,6 +2861,9 @@
       <c r="B224" s="1" t="str">
         <v/>
       </c>
+      <c r="C224" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="str">
@@ -2199,6 +2872,9 @@
       <c r="B225" s="1" t="str">
         <v/>
       </c>
+      <c r="C225" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="str">
@@ -2207,6 +2883,9 @@
       <c r="B226" s="1" t="str">
         <v/>
       </c>
+      <c r="C226" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="str">
@@ -2215,6 +2894,9 @@
       <c r="B227" s="1" t="str">
         <v/>
       </c>
+      <c r="C227" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="str">
@@ -2223,6 +2905,9 @@
       <c r="B228" s="1" t="str">
         <v/>
       </c>
+      <c r="C228" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="str">
@@ -2231,6 +2916,9 @@
       <c r="B229" s="1" t="str">
         <v/>
       </c>
+      <c r="C229" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="str">
@@ -2239,6 +2927,9 @@
       <c r="B230" s="1" t="str">
         <v/>
       </c>
+      <c r="C230" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="str">
@@ -2247,6 +2938,9 @@
       <c r="B231" s="1" t="str">
         <v/>
       </c>
+      <c r="C231" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="str">
@@ -2255,6 +2949,9 @@
       <c r="B232" s="1" t="str">
         <v/>
       </c>
+      <c r="C232" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="str">
@@ -2263,6 +2960,9 @@
       <c r="B233" s="1" t="str">
         <v/>
       </c>
+      <c r="C233" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="str">
@@ -2271,6 +2971,9 @@
       <c r="B234" s="1" t="str">
         <v/>
       </c>
+      <c r="C234" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="str">
@@ -2279,6 +2982,9 @@
       <c r="B235" s="1" t="str">
         <v/>
       </c>
+      <c r="C235" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="str">
@@ -2287,6 +2993,9 @@
       <c r="B236" s="1" t="str">
         <v/>
       </c>
+      <c r="C236" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="str">
@@ -2295,6 +3004,9 @@
       <c r="B237" s="1" t="str">
         <v/>
       </c>
+      <c r="C237" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="str">
@@ -2303,6 +3015,9 @@
       <c r="B238" s="1" t="str">
         <v/>
       </c>
+      <c r="C238" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="str">
@@ -2311,6 +3026,9 @@
       <c r="B239" s="1" t="str">
         <v/>
       </c>
+      <c r="C239" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="str">
@@ -2319,6 +3037,9 @@
       <c r="B240" s="1" t="str">
         <v/>
       </c>
+      <c r="C240" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="str">
@@ -2327,6 +3048,9 @@
       <c r="B241" s="1" t="str">
         <v/>
       </c>
+      <c r="C241" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="str">
@@ -2335,6 +3059,9 @@
       <c r="B242" s="1" t="str">
         <v/>
       </c>
+      <c r="C242" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="str">
@@ -2343,6 +3070,9 @@
       <c r="B243" s="1" t="str">
         <v/>
       </c>
+      <c r="C243" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="str">
@@ -2351,6 +3081,9 @@
       <c r="B244" s="1" t="str">
         <v/>
       </c>
+      <c r="C244" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="str">
@@ -2359,6 +3092,9 @@
       <c r="B245" s="1" t="str">
         <v/>
       </c>
+      <c r="C245" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="str">
@@ -2367,6 +3103,9 @@
       <c r="B246" s="1" t="str">
         <v/>
       </c>
+      <c r="C246" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="str">
@@ -2375,6 +3114,9 @@
       <c r="B247" s="1" t="str">
         <v/>
       </c>
+      <c r="C247" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="str">
@@ -2383,6 +3125,9 @@
       <c r="B248" s="1" t="str">
         <v/>
       </c>
+      <c r="C248" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="str">
@@ -2391,6 +3136,9 @@
       <c r="B249" s="1" t="str">
         <v/>
       </c>
+      <c r="C249" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="str">
@@ -2399,6 +3147,9 @@
       <c r="B250" s="1" t="str">
         <v/>
       </c>
+      <c r="C250" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="str">
@@ -2407,6 +3158,9 @@
       <c r="B251" s="1" t="str">
         <v/>
       </c>
+      <c r="C251" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="str">
@@ -2415,6 +3169,9 @@
       <c r="B252" s="1" t="str">
         <v/>
       </c>
+      <c r="C252" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="str">
@@ -2423,6 +3180,9 @@
       <c r="B253" s="1" t="str">
         <v/>
       </c>
+      <c r="C253" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="str">
@@ -2431,6 +3191,9 @@
       <c r="B254" s="1" t="str">
         <v/>
       </c>
+      <c r="C254" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="str">
@@ -2439,6 +3202,9 @@
       <c r="B255" s="1" t="str">
         <v/>
       </c>
+      <c r="C255" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="str">
@@ -2447,6 +3213,9 @@
       <c r="B256" s="1" t="str">
         <v/>
       </c>
+      <c r="C256" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="1" t="str">
@@ -2455,6 +3224,9 @@
       <c r="B257" s="1" t="str">
         <v/>
       </c>
+      <c r="C257" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="str">
@@ -2463,6 +3235,9 @@
       <c r="B258" s="1" t="str">
         <v/>
       </c>
+      <c r="C258" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="str">
@@ -2471,6 +3246,9 @@
       <c r="B259" s="1" t="str">
         <v/>
       </c>
+      <c r="C259" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="str">
@@ -2479,6 +3257,9 @@
       <c r="B260" s="1" t="str">
         <v/>
       </c>
+      <c r="C260" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="str">
@@ -2487,6 +3268,9 @@
       <c r="B261" s="1" t="str">
         <v/>
       </c>
+      <c r="C261" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="str">
@@ -2495,6 +3279,9 @@
       <c r="B262" s="1" t="str">
         <v/>
       </c>
+      <c r="C262" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="str">
@@ -2503,6 +3290,9 @@
       <c r="B263" s="1" t="str">
         <v/>
       </c>
+      <c r="C263" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="str">
@@ -2511,6 +3301,9 @@
       <c r="B264" s="1" t="str">
         <v/>
       </c>
+      <c r="C264" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="str">
@@ -2519,6 +3312,9 @@
       <c r="B265" s="1" t="str">
         <v/>
       </c>
+      <c r="C265" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="str">
@@ -2527,6 +3323,9 @@
       <c r="B266" s="1" t="str">
         <v/>
       </c>
+      <c r="C266" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="str">
@@ -2535,6 +3334,9 @@
       <c r="B267" s="1" t="str">
         <v/>
       </c>
+      <c r="C267" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="str">
@@ -2543,6 +3345,9 @@
       <c r="B268" s="1" t="str">
         <v/>
       </c>
+      <c r="C268" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="str">
@@ -2551,6 +3356,9 @@
       <c r="B269" s="1" t="str">
         <v/>
       </c>
+      <c r="C269" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="str">
@@ -2559,6 +3367,9 @@
       <c r="B270" s="1" t="str">
         <v/>
       </c>
+      <c r="C270" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="str">
@@ -2567,6 +3378,9 @@
       <c r="B271" s="1" t="str">
         <v/>
       </c>
+      <c r="C271" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="str">
@@ -2575,6 +3389,9 @@
       <c r="B272" s="1" t="str">
         <v/>
       </c>
+      <c r="C272" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="str">
@@ -2583,6 +3400,9 @@
       <c r="B273" s="1" t="str">
         <v/>
       </c>
+      <c r="C273" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="str">
@@ -2591,6 +3411,9 @@
       <c r="B274" s="1" t="str">
         <v/>
       </c>
+      <c r="C274" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="str">
@@ -2599,6 +3422,9 @@
       <c r="B275" s="1" t="str">
         <v/>
       </c>
+      <c r="C275" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="str">
@@ -2607,6 +3433,9 @@
       <c r="B276" s="1" t="str">
         <v/>
       </c>
+      <c r="C276" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="str">
@@ -2615,6 +3444,9 @@
       <c r="B277" s="1" t="str">
         <v/>
       </c>
+      <c r="C277" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="str">
@@ -2623,6 +3455,9 @@
       <c r="B278" s="1" t="str">
         <v/>
       </c>
+      <c r="C278" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="str">
@@ -2631,6 +3466,9 @@
       <c r="B279" s="1" t="str">
         <v/>
       </c>
+      <c r="C279" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="str">
@@ -2639,6 +3477,9 @@
       <c r="B280" s="1" t="str">
         <v/>
       </c>
+      <c r="C280" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="str">
@@ -2647,6 +3488,9 @@
       <c r="B281" s="1" t="str">
         <v/>
       </c>
+      <c r="C281" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="str">
@@ -2655,6 +3499,9 @@
       <c r="B282" s="1" t="str">
         <v/>
       </c>
+      <c r="C282" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="str">
@@ -2663,6 +3510,9 @@
       <c r="B283" s="1" t="str">
         <v/>
       </c>
+      <c r="C283" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="str">
@@ -2671,6 +3521,9 @@
       <c r="B284" s="1" t="str">
         <v/>
       </c>
+      <c r="C284" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="str">
@@ -2679,6 +3532,9 @@
       <c r="B285" s="1" t="str">
         <v/>
       </c>
+      <c r="C285" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="str">
@@ -2687,6 +3543,9 @@
       <c r="B286" s="1" t="str">
         <v/>
       </c>
+      <c r="C286" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="str">
@@ -2695,6 +3554,9 @@
       <c r="B287" s="1" t="str">
         <v/>
       </c>
+      <c r="C287" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="str">
@@ -2703,6 +3565,9 @@
       <c r="B288" s="1" t="str">
         <v/>
       </c>
+      <c r="C288" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="str">
@@ -2711,6 +3576,9 @@
       <c r="B289" s="1" t="str">
         <v/>
       </c>
+      <c r="C289" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="str">
@@ -2719,6 +3587,9 @@
       <c r="B290" s="1" t="str">
         <v/>
       </c>
+      <c r="C290" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="str">
@@ -2727,6 +3598,9 @@
       <c r="B291" s="1" t="str">
         <v/>
       </c>
+      <c r="C291" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="str">
@@ -2735,6 +3609,9 @@
       <c r="B292" s="1" t="str">
         <v/>
       </c>
+      <c r="C292" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="str">
@@ -2743,6 +3620,9 @@
       <c r="B293" s="1" t="str">
         <v/>
       </c>
+      <c r="C293" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="str">
@@ -2751,6 +3631,9 @@
       <c r="B294" s="1" t="str">
         <v/>
       </c>
+      <c r="C294" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="str">
@@ -2759,6 +3642,9 @@
       <c r="B295" s="1" t="str">
         <v/>
       </c>
+      <c r="C295" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="str">
@@ -2767,6 +3653,9 @@
       <c r="B296" s="1" t="str">
         <v/>
       </c>
+      <c r="C296" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="str">
@@ -2775,6 +3664,9 @@
       <c r="B297" s="1" t="str">
         <v/>
       </c>
+      <c r="C297" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="str">
@@ -2783,6 +3675,9 @@
       <c r="B298" s="1" t="str">
         <v/>
       </c>
+      <c r="C298" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="str">
@@ -2791,6 +3686,9 @@
       <c r="B299" s="1" t="str">
         <v/>
       </c>
+      <c r="C299" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="str">
@@ -2799,6 +3697,9 @@
       <c r="B300" s="1" t="str">
         <v/>
       </c>
+      <c r="C300" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="str">
@@ -2807,10 +3708,145 @@
       <c r="B301" s="1" t="str">
         <v/>
       </c>
+      <c r="C301" s="1" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B301"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C301"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PETUNJUK PENGISIAN — DUDI (Mitra PKL)</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Kolom</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Wajib?</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Penjelasan</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>nama_usaha</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Wajib</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Nama lengkap usaha atau perusahaan mitra PKL. Nama ini menjadi identitas login DUDI.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>nama_penanggung_jawab</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Wajib</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nama penanggung jawab dari pihak usaha.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>kode_program</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Kode program keahlian yang menaungi DUDI ini (mis. TKJ, AKL). Menautkan DUDI ke Kaprodi program tersebut sehingga muncul sebagai mitra di dashboard Kaprodi. Kosongkan bila DUDI lintas program.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>PENTING</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>•</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v>DUDI login menggunakan nama usaha (bukan NIK). Sistem otomatis membuat kode login dari nama usaha.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>•</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v>kode_program harus sudah ada di langkah Program Keahlian. Bila diisi tapi kode tidak dikenal, baris tersebut ditolak.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>•</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v>Upload ulang file yang sama akan memperbarui nama usaha, penanggung jawab, dan program.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>